<commit_message>
minor changes to run as a service
</commit_message>
<xml_diff>
--- a/state table.xlsx
+++ b/state table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\protonThreaded\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AD7F237-E6D5-4323-954D-FE4CC1F824D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E56B4700-EEAA-4778-8785-6EC443FFF253}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="5685" windowWidth="18240" windowHeight="28320" xr2:uid="{737C3618-456B-49FB-A30C-D008677A7A19}"/>
   </bookViews>
@@ -98,9 +98,6 @@
     <t>Flashing Blue</t>
   </si>
   <si>
-    <t>Flashing Orange</t>
-  </si>
-  <si>
     <t>No logs are being saved. The logger is is unable to save to thumb drive or backup location</t>
   </si>
   <si>
@@ -120,6 +117,9 @@
   </si>
   <si>
     <t>Line running, thumb drive OK, saving logs to thumb drive</t>
+  </si>
+  <si>
+    <t>Flashing Magenta</t>
   </si>
 </sst>
 </file>
@@ -151,12 +151,42 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC00000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -186,21 +216,36 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -218,6 +263,55 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>28575</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>26846</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1104900</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>86650</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CEE68078-4BEB-D976-5A79-6AA9F54F95E7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="238125" y="6580046"/>
+          <a:ext cx="5915025" cy="1583804"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -537,181 +631,175 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDB36707-E540-419C-B25B-E37827A81E6E}">
-  <dimension ref="C2:E18"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="B2:H10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="10" style="1" customWidth="1"/>
-    <col min="4" max="4" width="32.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="33.42578125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="3.140625" customWidth="1"/>
+    <col min="2" max="2" width="9.7109375" style="1" customWidth="1"/>
+    <col min="3" max="4" width="16.7109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="3" customWidth="1"/>
+    <col min="6" max="6" width="9.7109375" customWidth="1"/>
+    <col min="7" max="8" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="3:5" ht="21" x14ac:dyDescent="0.25">
-      <c r="C2" s="2" t="s">
+    <row r="2" spans="2:8" ht="21" x14ac:dyDescent="0.25">
+      <c r="B2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="F2" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
     </row>
-    <row r="3" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C3" s="3" t="s">
+    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="D3" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="F3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="4" spans="3:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="B4" s="3" t="s">
+        <v>7</v>
+      </c>
       <c r="C4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="G4" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="H4" s="5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C5" s="5" t="s">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
+      <c r="F5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
     </row>
-    <row r="6" spans="3:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="C6" s="5" t="s">
+    <row r="6" spans="2:8" ht="90" x14ac:dyDescent="0.25">
+      <c r="B6" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="C6" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="D6" s="3" t="s">
         <v>10</v>
       </c>
+      <c r="F6" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>20</v>
+      </c>
     </row>
-    <row r="7" spans="3:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="C7" s="5" t="s">
+    <row r="7" spans="2:8" ht="75" x14ac:dyDescent="0.25">
+      <c r="B7" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="C7" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="D7" s="3" t="s">
         <v>13</v>
       </c>
+      <c r="F7" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="8" spans="3:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="C8" s="5" t="s">
+    <row r="8" spans="2:8" ht="105" x14ac:dyDescent="0.25">
+      <c r="B8" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="C8" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="D8" s="3" t="s">
         <v>16</v>
       </c>
+      <c r="F8" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H8" s="5"/>
     </row>
-    <row r="10" spans="3:5" ht="21" x14ac:dyDescent="0.25">
-      <c r="C10" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
+    <row r="9" spans="2:8" ht="90" x14ac:dyDescent="0.25">
+      <c r="F9" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>16</v>
+      </c>
     </row>
-    <row r="11" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C11" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12" spans="3:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="C12" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="13" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C13" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-    </row>
-    <row r="14" spans="3:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="C14" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="15" spans="3:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="C15" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="16" spans="3:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="C16" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="E16" s="4"/>
-    </row>
-    <row r="17" spans="3:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="C17" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D17" s="5" t="s">
+    <row r="10" spans="2:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="F10" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G10" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="E17" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="18" spans="3:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="C18" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="E18" s="4"/>
+      <c r="H10" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="C2:E2"/>
+    <mergeCell ref="H7:H8"/>
+    <mergeCell ref="H9:H10"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="C4:C5"/>
     <mergeCell ref="D4:D5"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="D12:D13"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="G4:G5"/>
+    <mergeCell ref="H4:H5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup scale="97" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>